<commit_message>
news: daily briefing 2026-10-08
</commit_message>
<xml_diff>
--- a/public-site/news/downloads/mfds-drug-supply-issues.xlsx
+++ b/public-site/news/downloads/mfds-drug-supply-issues.xlsx
@@ -139,7 +139,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K1"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -211,72 +211,15 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">스카이바리셀라주(수두생바이러스백신)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">에스케이바이오사이언스(주)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-12</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">공정 최적화에 따른 허가 변경이 필요하여 변경허가를 신청하였으며, 변경허가 승인 전까지 일시적으로 생산을 중단합니다.</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">타 사의 수두백신이 공급중인 바, 환자 치료에 큰 영향을 미치지 않을 것으로 판단됩니다. 다만, 해당 품목의 빠른 공급 안정화를 도모하여 장기적으로 공급에 영향을 미치지 않도록 만전을 기하겠습니다.</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">허가 변경이 완료되는 대로 공급 정상화될수 있도록 할 예정이며, 이후 공급에 차질이 없도록 하겠습니다.​</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2027-03-18</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-12</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10000</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8800564000520</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K2"/>
+  <autoFilter ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="18"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -462,236 +405,8 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-08</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">옥시콘틴서방정80mg(옥시코돈염산염)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">한국먼디파마 유한회사</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-30</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">입고된 수량에 대비하여 시장 출고량이 현저히 높아짐에 따라, 국내 창고 물량의 빠른 소진 및 일시적인 국내 시장 공급 어려움이 예상되었습니다. 이에 따라, 해외 완제의약품 수입을 빠르게 진행하고자 하였으나, 현지 완제의약품 출고가 지연되고 있습니다.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">옥시콘틴서방정의 일시적인 부족이 환자 치료에 미치는 영향은 제한적일 것으로 사료됩니다. 시장에는 옥시콘틴과 동일한 유효성분을 함유한 제네릭 의약품이 이미 유통되고 있습니다.</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">빠른 시일 내 공급정상화가 되도록 노력하겠습니다.</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-11-02</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-03</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3630</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8806780001631</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-08</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">옥시콘틴서방정40밀리그램(옥시코돈염산염)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">한국먼디파마 유한회사</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2027-01-29</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">입고된 수량에 대비하여 시장 출고량이 현저히 높아짐에 따라, 국내 창고 물량의 빠른 소진 및 일시적인 국내 시장 공급 어려움이 예상되었습니다. 이에 따라, 해외 완제의약품 수입을 빠르게 진행하고자 하였으나, 현지 완제의약품 출고가 지연되고 있습니다.</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">옥시콘틴서방정의 일시적인 부족이 환자 치료에 미치는 영향은 제한적일 것으로 사료됩니다. 시장에는 옥시콘틴과 동일한 유효성분을 함유한 제네릭 의약품이 이미 유통되고 있습니다.</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">빠른 시일 내 공급정상화가 되도록 노력하겠습니다.</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2027-03-01</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-20</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12090</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8806780001136</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-08</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">옥시콘틴서방정20밀리그램(옥시코돈염산염)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">한국먼디파마 유한회사</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-11-16</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">입고된 수량에 대비하여 시장 출고량이 현저히 높아짐에 따라, 국내 창고 물량의 빠른 소진 및 일시적인 국내 시장 공급 어려움이 예상되었습니다. 이에 따라, 해외 완제의약품 수입을 빠르게 진행하고자 하였으나, 현지 완제의약품 출고가 지연되고 있습니다.</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">옥시콘틴서방정의 일시적인 부족이 환자 치료에 미치는 영향은 제한적일 것으로 사료됩니다. 시장에는 옥시콘틴과 동일한 유효성분을 함유한 제네릭 의약품이 이미 유통되고 있습니다.</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">빠른 시일 내 공급정상화가 되도록 노력하겠습니다.</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2027-03-01</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-20</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">19500</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8806780001037</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-08</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">옥시콘틴서방정10밀리그램(옥시코돈염산염)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">한국먼디파마 유한회사</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2027-02-15</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">입고된 수량에 대비하여 시장 출고량이 현저히 높아짐에 따라, 국내 창고 물량의 빠른 소진 및 일시적인 국내 시장 공급 어려움이 예상되었습니다. 이에 따라, 해외 완제의약품 수입을 빠르게 진행하고자 하였으나, 현지 완제의약품 출고가 지연되고 있습니다.</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">옥시콘틴서방정의 일시적인 부족이 환자 치료에 미치는 영향은 제한적일 것으로 사료됩니다. 시장에는 옥시콘틴과 동일한 유효성분을 함유한 제네릭 의약품이 이미 유통되고 있습니다.</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">빠른 시일 내 공급정상화가 되도록 노력하겠습니다.</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2027-03-01</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-20</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30000</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8806780000931</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K7"/>
+  <autoFilter ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="18"/>
 </worksheet>
 </file>
@@ -1321,7 +1036,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-07-01</t>
+          <t xml:space="preserve">2028-12-31</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1378,7 +1093,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-07-01</t>
+          <t xml:space="preserve">2028-12-31</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">

</xml_diff>

<commit_message>
news: daily briefing 2026-10-15
</commit_message>
<xml_diff>
--- a/public-site/news/downloads/mfds-drug-supply-issues.xlsx
+++ b/public-site/news/downloads/mfds-drug-supply-issues.xlsx
@@ -219,7 +219,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K2"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -348,65 +348,8 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-15</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">엔독산주500mg(시클로포스파미드)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">부광약품(주)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-12</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">수입 후 실시한 품질시험(무균시험) 기준일탈에 따른 출하 보류(미출하)</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">동일 성분 대체제는 없으며, 시클로포스파미드는 7개 적응증에 대한 단독 또는 병용 항암요법에 포함되어 있습니다. 환자별로 적합한 치료 요법은 환자의 개별 특성에 따른 의료 전문가의 판단이 필요하나, 「암환자에게 처방･투여하는 약제에 대한 요양급여의 적용기준 및 방법에 관한 세부사항」을 고려할 때, 시클로포스파미드 주사제가 포함된 치료 요법의 대체와 관련하여 첨부드린 자료를 참고할 수 있을 것으로 사료됩니다.</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10월 중순 입고예정으로 입고 즉시 최우선으로 품질시험을 진행할 예정이며, 11월 내에 공급 부족이 해소될 것으로 예상됩니다.</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-11-09</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-15</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">19,609</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8806422016719</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K3"/>
+  <autoFilter ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="18"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
news: daily briefing 2026-10-23
</commit_message>
<xml_diff>
--- a/public-site/news/downloads/mfds-drug-supply-issues.xlsx
+++ b/public-site/news/downloads/mfds-drug-supply-issues.xlsx
@@ -139,7 +139,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K2"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -268,65 +268,8 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-16</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">스카이바리셀라주(수두생바이러스백신)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">에스케이바이오사이언스(주)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-19</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">공정 최적화에 따른 허가 변경이 필요하여 변경허가를 신청하였으며, 변경허가 승인 전까지 일시적으로 생산을 중단합니다.</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">타 사의 수두백신이 공급중인 바, 환자 치료에 큰 영향을 미치지 않을 것으로 판단됩니다. 다만, 해당 품목의 빠른 공급 안정화를 도모하여 장기적으로 공급에 영향을 미치지 않도록 만전을 기하겠습니다.</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">허가 변경이 완료되는 대로 공급 정상화될수 있도록 할 예정이며, 이후 공급에 차질이 없도록 하겠습니다.​</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2027-03-18</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-19</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8800564000506,8806447046203,8800564000513,8806447046227,8800564000520,8806447046210,8800564000537</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K3"/>
+  <autoFilter ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="18"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
news: daily briefing 2026-10-25
</commit_message>
<xml_diff>
--- a/public-site/news/downloads/mfds-drug-supply-issues.xlsx
+++ b/public-site/news/downloads/mfds-drug-supply-issues.xlsx
@@ -139,7 +139,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -214,62 +214,119 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t xml:space="preserve">2026-10-23</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">스카이바리셀라주(수두생바이러스백신)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">에스케이바이오사이언스(주)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-23</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">공정 최적화에 따른 허가 변경이 필요하여 변경허가를 신청하였으며, 변경허가 승인 전까지 일시적으로 생산을 중단합니다.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">타 사의 수두백신이 공급중인 바, 환자 치료에 큰 영향을 미치지 않을 것으로 판단됩니다. 다만, 해당 품목의 빠른 공급 안정화를 도모하여 장기적으로 공급에 영향을 미치지 않도록 만전을 기하겠습니다.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">허가 변경이 완료되는 대로 공급 정상화될수 있도록 할 예정이며, 이후 공급에 차질이 없도록 하겠습니다.​</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2027-03-18</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-23</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8800564000506,8806447046203,8800564000513,8806447046227,8800564000520,8806447046210,8800564000537</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t xml:space="preserve">2026-10-20</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t xml:space="preserve">유니레이프리필드주사</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t xml:space="preserve">동국제약(주)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t xml:space="preserve">2027-04-20</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t xml:space="preserve">원료 수급 문제 - 중국 당국의 정부 수출 통제 조치로 인해 산화가돌리늄의 출발물질(희토류 금속) 등에 대한 수출 허가가 승인되지 않고 있음. - 산화가돌리늄 생산 : 출발물질 등의 수급 이슈로 인해 산화가돌리늄의 제조사에서 생산 차질이 발생 - 향후 전망 : 중국 당국의 수출 허가 승인 시점이 불확실하여 향후 납품 지연 예상</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t xml:space="preserve">‘유니레이프리필드주사’는 국내 가도테레이트메글루민 시장의 약 38%를 담당하는 유일한 국내 생산 조영제입니다. 공급이 부족할 시 국내에서 생산되는 조영제의 공급 기반을 축소하고 수입 제품에 대한 의존도를 심화시키는 결과를 초래할 수 있습니다. 당사는 유니레이 공급 부족에 따른 의료현장의 영향을 최소화하기 위해 생산 정상화를 위한 원료 확보를 최우선적으로 추진하고 있습니다.</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t xml:space="preserve">1. 기존 제조처 공급 정상화 추진 기존 제조처에 원료 수급 및 생산 현황을 지속적으로 확인하고, 중국 당국의 수출 허가 승인 진행 상황을 주기적으로 점검 2. 신규 제조처 발굴 및 공급처 다변화 기존 제조처의 공급 차질에 대응하기 위해 산화가돌리늄을 안정적으로 공급할 수 있는 신규 제조처 발굴 및 수배 추진 신규 제조처의 원료 수급 안정성, 생산능력, 품질관리 체계 및 공급 가능 일정 등을 종합적으로 검토 3. 신규 제조처 품질 확보 및 공급 적합성 검증 신규 제조처 확보 후 원료 및 제조 공정의 차이를 고려한 제제연구를 실시하여 기존 제품과의 동등성 및 품질 적합성 검토 시험 생산을 통해 제조공정의 재현성, 제품 품질 및 주요 품질 특성에 대한 평가 실시 4. 공급 부족 대응 및 정상화 관리 기존 제조처의 공급 정상화 추진 현황과 신규 제조처 확보 및 품질 검증 진행 상활을 지속적으로 모니터링 공급 주족 예상 기간 및 확보 가능 물량을 고려하여 재고 현황과 수요를 점검하고, 공급 공백 최소화 방안 마련</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t xml:space="preserve">2028-06-30</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-20</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t xml:space="preserve">8806534027825,8806534027924,8806534028020</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K2"/>
+  <autoFilter ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="18"/>
 </worksheet>
 </file>
@@ -351,47 +408,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20</t>
+          <t xml:space="preserve">2026-10-23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">유니레이프리필드주사</t>
+          <t xml:space="preserve">스카이바리셀라주(수두생바이러스백신)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">동국제약(주)</t>
+          <t xml:space="preserve">에스케이바이오사이언스(주)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-04-20</t>
+          <t xml:space="preserve">2026-10-23</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">원료 수급 문제 - 중국 당국의 정부 수출 통제 조치로 인해 산화가돌리늄의 출발물질(희토류 금속) 등에 대한 수출 허가가 승인되지 않고 있음. - 산화가돌리늄 생산 : 출발물질 등의 수급 이슈로 인해 산화가돌리늄의 제조사에서 생산 차질이 발생 - 향후 전망 : 중국 당국의 수출 허가 승인 시점이 불확실하여 향후 납품 지연 예상</t>
+          <t xml:space="preserve">공정 최적화에 따른 허가 변경이 필요하여 변경허가를 신청하였으며, 변경허가 승인 전까지 일시적으로 생산을 중단합니다.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">‘유니레이프리필드주사’는 국내 가도테레이트메글루민 시장의 약 38%를 담당하는 유일한 국내 생산 조영제입니다. 공급이 부족할 시 국내에서 생산되는 조영제의 공급 기반을 축소하고 수입 제품에 대한 의존도를 심화시키는 결과를 초래할 수 있습니다. 당사는 유니레이 공급 부족에 따른 의료현장의 영향을 최소화하기 위해 생산 정상화를 위한 원료 확보를 최우선적으로 추진하고 있습니다.</t>
+          <t xml:space="preserve">타 사의 수두백신이 공급중인 바, 환자 치료에 큰 영향을 미치지 않을 것으로 판단됩니다. 다만, 해당 품목의 빠른 공급 안정화를 도모하여 장기적으로 공급에 영향을 미치지 않도록 만전을 기하겠습니다.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. 기존 제조처 공급 정상화 추진 기존 제조처에 원료 수급 및 생산 현황을 지속적으로 확인하고, 중국 당국의 수출 허가 승인 진행 상황을 주기적으로 점검 2. 신규 제조처 발굴 및 공급처 다변화 기존 제조처의 공급 차질에 대응하기 위해 산화가돌리늄을 안정적으로 공급할 수 있는 신규 제조처 발굴 및 수배 추진 신규 제조처의 원료 수급 안정성, 생산능력, 품질관리 체계 및 공급 가능 일정 등을 종합적으로 검토 3. 신규 제조처 품질 확보 및 공급 적합성 검증 신규 제조처 확보 후 원료 및 제조 공정의 차이를 고려한 제제연구를 실시하여 기존 제품과의 동등성 및 품질 적합성 검토 시험 생산을 통해 제조공정의 재현성, 제품 품질 및 주요 품질 특성에 대한 평가 실시 4. 공급 부족 대응 및 정상화 관리 기존 제조처의 공급 정상화 추진 현황과 신규 제조처 확보 및 품질 검증 진행 상활을 지속적으로 모니터링 공급 주족 예상 기간 및 확보 가능 물량을 고려하여 재고 현황과 수요를 점검하고, 공급 공백 최소화 방안 마련</t>
+          <t xml:space="preserve">허가 변경이 완료되는 대로 공급 정상화될수 있도록 할 예정이며, 이후 공급에 차질이 없도록 하겠습니다.​</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2028-06-30</t>
+          <t xml:space="preserve">2027-03-18</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20</t>
+          <t xml:space="preserve">2026-10-23</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -401,54 +458,54 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8806534027825,8806534027924,8806534028020</t>
+          <t xml:space="preserve">8800564000506,8806447046203,8800564000513,8806447046227,8800564000520,8806447046210,8800564000537</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-16</t>
+          <t xml:space="preserve">2026-10-20</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">스카이바리셀라주(수두생바이러스백신)</t>
+          <t xml:space="preserve">유니레이프리필드주사</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">에스케이바이오사이언스(주)</t>
+          <t xml:space="preserve">동국제약(주)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-19</t>
+          <t xml:space="preserve">2027-04-20</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">공정 최적화에 따른 허가 변경이 필요하여 변경허가를 신청하였으며, 변경허가 승인 전까지 일시적으로 생산을 중단합니다.</t>
+          <t xml:space="preserve">원료 수급 문제 - 중국 당국의 정부 수출 통제 조치로 인해 산화가돌리늄의 출발물질(희토류 금속) 등에 대한 수출 허가가 승인되지 않고 있음. - 산화가돌리늄 생산 : 출발물질 등의 수급 이슈로 인해 산화가돌리늄의 제조사에서 생산 차질이 발생 - 향후 전망 : 중국 당국의 수출 허가 승인 시점이 불확실하여 향후 납품 지연 예상</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">타 사의 수두백신이 공급중인 바, 환자 치료에 큰 영향을 미치지 않을 것으로 판단됩니다. 다만, 해당 품목의 빠른 공급 안정화를 도모하여 장기적으로 공급에 영향을 미치지 않도록 만전을 기하겠습니다.</t>
+          <t xml:space="preserve">‘유니레이프리필드주사’는 국내 가도테레이트메글루민 시장의 약 38%를 담당하는 유일한 국내 생산 조영제입니다. 공급이 부족할 시 국내에서 생산되는 조영제의 공급 기반을 축소하고 수입 제품에 대한 의존도를 심화시키는 결과를 초래할 수 있습니다. 당사는 유니레이 공급 부족에 따른 의료현장의 영향을 최소화하기 위해 생산 정상화를 위한 원료 확보를 최우선적으로 추진하고 있습니다.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">허가 변경이 완료되는 대로 공급 정상화될수 있도록 할 예정이며, 이후 공급에 차질이 없도록 하겠습니다.​</t>
+          <t xml:space="preserve">1. 기존 제조처 공급 정상화 추진 기존 제조처에 원료 수급 및 생산 현황을 지속적으로 확인하고, 중국 당국의 수출 허가 승인 진행 상황을 주기적으로 점검 2. 신규 제조처 발굴 및 공급처 다변화 기존 제조처의 공급 차질에 대응하기 위해 산화가돌리늄을 안정적으로 공급할 수 있는 신규 제조처 발굴 및 수배 추진 신규 제조처의 원료 수급 안정성, 생산능력, 품질관리 체계 및 공급 가능 일정 등을 종합적으로 검토 3. 신규 제조처 품질 확보 및 공급 적합성 검증 신규 제조처 확보 후 원료 및 제조 공정의 차이를 고려한 제제연구를 실시하여 기존 제품과의 동등성 및 품질 적합성 검토 시험 생산을 통해 제조공정의 재현성, 제품 품질 및 주요 품질 특성에 대한 평가 실시 4. 공급 부족 대응 및 정상화 관리 기존 제조처의 공급 정상화 추진 현황과 신규 제조처 확보 및 품질 검증 진행 상활을 지속적으로 모니터링 공급 주족 예상 기간 및 확보 가능 물량을 고려하여 재고 현황과 수요를 점검하고, 공급 공백 최소화 방안 마련</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-03-18</t>
+          <t xml:space="preserve">2028-06-30</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-19</t>
+          <t xml:space="preserve">2026-10-20</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -458,7 +515,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8800564000506,8806447046203,8800564000513,8806447046227,8800564000520,8806447046210,8800564000537</t>
+          <t xml:space="preserve">8806534027825,8806534027924,8806534028020</t>
         </is>
       </c>
     </row>
@@ -545,47 +602,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20</t>
+          <t xml:space="preserve">2026-10-23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">유니레이프리필드주사</t>
+          <t xml:space="preserve">스카이바리셀라주(수두생바이러스백신)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">동국제약(주)</t>
+          <t xml:space="preserve">에스케이바이오사이언스(주)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-04-20</t>
+          <t xml:space="preserve">2026-10-23</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">원료 수급 문제 - 중국 당국의 정부 수출 통제 조치로 인해 산화가돌리늄의 출발물질(희토류 금속) 등에 대한 수출 허가가 승인되지 않고 있음. - 산화가돌리늄 생산 : 출발물질 등의 수급 이슈로 인해 산화가돌리늄의 제조사에서 생산 차질이 발생 - 향후 전망 : 중국 당국의 수출 허가 승인 시점이 불확실하여 향후 납품 지연 예상</t>
+          <t xml:space="preserve">공정 최적화에 따른 허가 변경이 필요하여 변경허가를 신청하였으며, 변경허가 승인 전까지 일시적으로 생산을 중단합니다.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">‘유니레이프리필드주사’는 국내 가도테레이트메글루민 시장의 약 38%를 담당하는 유일한 국내 생산 조영제입니다. 공급이 부족할 시 국내에서 생산되는 조영제의 공급 기반을 축소하고 수입 제품에 대한 의존도를 심화시키는 결과를 초래할 수 있습니다. 당사는 유니레이 공급 부족에 따른 의료현장의 영향을 최소화하기 위해 생산 정상화를 위한 원료 확보를 최우선적으로 추진하고 있습니다.</t>
+          <t xml:space="preserve">타 사의 수두백신이 공급중인 바, 환자 치료에 큰 영향을 미치지 않을 것으로 판단됩니다. 다만, 해당 품목의 빠른 공급 안정화를 도모하여 장기적으로 공급에 영향을 미치지 않도록 만전을 기하겠습니다.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. 기존 제조처 공급 정상화 추진 기존 제조처에 원료 수급 및 생산 현황을 지속적으로 확인하고, 중국 당국의 수출 허가 승인 진행 상황을 주기적으로 점검 2. 신규 제조처 발굴 및 공급처 다변화 기존 제조처의 공급 차질에 대응하기 위해 산화가돌리늄을 안정적으로 공급할 수 있는 신규 제조처 발굴 및 수배 추진 신규 제조처의 원료 수급 안정성, 생산능력, 품질관리 체계 및 공급 가능 일정 등을 종합적으로 검토 3. 신규 제조처 품질 확보 및 공급 적합성 검증 신규 제조처 확보 후 원료 및 제조 공정의 차이를 고려한 제제연구를 실시하여 기존 제품과의 동등성 및 품질 적합성 검토 시험 생산을 통해 제조공정의 재현성, 제품 품질 및 주요 품질 특성에 대한 평가 실시 4. 공급 부족 대응 및 정상화 관리 기존 제조처의 공급 정상화 추진 현황과 신규 제조처 확보 및 품질 검증 진행 상활을 지속적으로 모니터링 공급 주족 예상 기간 및 확보 가능 물량을 고려하여 재고 현황과 수요를 점검하고, 공급 공백 최소화 방안 마련</t>
+          <t xml:space="preserve">허가 변경이 완료되는 대로 공급 정상화될수 있도록 할 예정이며, 이후 공급에 차질이 없도록 하겠습니다.​</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2028-06-30</t>
+          <t xml:space="preserve">2027-03-18</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20</t>
+          <t xml:space="preserve">2026-10-23</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -595,54 +652,54 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8806534027825,8806534027924,8806534028020</t>
+          <t xml:space="preserve">8800564000506,8806447046203,8800564000513,8806447046227,8800564000520,8806447046210,8800564000537</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-16</t>
+          <t xml:space="preserve">2026-10-20</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">스카이바리셀라주(수두생바이러스백신)</t>
+          <t xml:space="preserve">유니레이프리필드주사</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">에스케이바이오사이언스(주)</t>
+          <t xml:space="preserve">동국제약(주)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-19</t>
+          <t xml:space="preserve">2027-04-20</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">공정 최적화에 따른 허가 변경이 필요하여 변경허가를 신청하였으며, 변경허가 승인 전까지 일시적으로 생산을 중단합니다.</t>
+          <t xml:space="preserve">원료 수급 문제 - 중국 당국의 정부 수출 통제 조치로 인해 산화가돌리늄의 출발물질(희토류 금속) 등에 대한 수출 허가가 승인되지 않고 있음. - 산화가돌리늄 생산 : 출발물질 등의 수급 이슈로 인해 산화가돌리늄의 제조사에서 생산 차질이 발생 - 향후 전망 : 중국 당국의 수출 허가 승인 시점이 불확실하여 향후 납품 지연 예상</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">타 사의 수두백신이 공급중인 바, 환자 치료에 큰 영향을 미치지 않을 것으로 판단됩니다. 다만, 해당 품목의 빠른 공급 안정화를 도모하여 장기적으로 공급에 영향을 미치지 않도록 만전을 기하겠습니다.</t>
+          <t xml:space="preserve">‘유니레이프리필드주사’는 국내 가도테레이트메글루민 시장의 약 38%를 담당하는 유일한 국내 생산 조영제입니다. 공급이 부족할 시 국내에서 생산되는 조영제의 공급 기반을 축소하고 수입 제품에 대한 의존도를 심화시키는 결과를 초래할 수 있습니다. 당사는 유니레이 공급 부족에 따른 의료현장의 영향을 최소화하기 위해 생산 정상화를 위한 원료 확보를 최우선적으로 추진하고 있습니다.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">허가 변경이 완료되는 대로 공급 정상화될수 있도록 할 예정이며, 이후 공급에 차질이 없도록 하겠습니다.​</t>
+          <t xml:space="preserve">1. 기존 제조처 공급 정상화 추진 기존 제조처에 원료 수급 및 생산 현황을 지속적으로 확인하고, 중국 당국의 수출 허가 승인 진행 상황을 주기적으로 점검 2. 신규 제조처 발굴 및 공급처 다변화 기존 제조처의 공급 차질에 대응하기 위해 산화가돌리늄을 안정적으로 공급할 수 있는 신규 제조처 발굴 및 수배 추진 신규 제조처의 원료 수급 안정성, 생산능력, 품질관리 체계 및 공급 가능 일정 등을 종합적으로 검토 3. 신규 제조처 품질 확보 및 공급 적합성 검증 신규 제조처 확보 후 원료 및 제조 공정의 차이를 고려한 제제연구를 실시하여 기존 제품과의 동등성 및 품질 적합성 검토 시험 생산을 통해 제조공정의 재현성, 제품 품질 및 주요 품질 특성에 대한 평가 실시 4. 공급 부족 대응 및 정상화 관리 기존 제조처의 공급 정상화 추진 현황과 신규 제조처 확보 및 품질 검증 진행 상활을 지속적으로 모니터링 공급 주족 예상 기간 및 확보 가능 물량을 고려하여 재고 현황과 수요를 점검하고, 공급 공백 최소화 방안 마련</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2027-03-18</t>
+          <t xml:space="preserve">2028-06-30</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-19</t>
+          <t xml:space="preserve">2026-10-20</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -652,7 +709,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8800564000506,8806447046203,8800564000513,8806447046227,8800564000520,8806447046210,8800564000537</t>
+          <t xml:space="preserve">8806534027825,8806534027924,8806534028020</t>
         </is>
       </c>
     </row>

</xml_diff>